<commit_message>
docs(vacaciones): hoja de la junta lista para llenar: guía, preguntas con opciones y personal con ejemplo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rsis6J1oMR6Czvco8XtVk
</commit_message>
<xml_diff>
--- a/docs/vacaciones/junta-montellano.xlsx
+++ b/docs/vacaciones/junta-montellano.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Altas y correcciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preguntas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Guía de la junta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Preguntas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Personal" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,10 +31,27 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001A3B70"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A3B70"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00888888"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -43,8 +63,23 @@
         <fgColor rgb="001A3B70"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F6FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -52,19 +87,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D4DC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D4DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D4DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D4DC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,71 +487,176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Acción</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Nombre (APELLIDOS NOMBRES)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Fecha de ingreso (dd/mm/aaaa)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Correo corporativo</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Puesto</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Área</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>No. de empleado</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Jefe directo (nombre)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Notas</t>
+          <t>Junta con Jesús Montellano — Vacaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: salir con fecha de arranque y con Jesús usando la plataforma él mismo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Qué hacer</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>¿Listo?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>ANTES</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Darle la bandera "Vacaciones RH" en /admin/usuarios</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>ANTES</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Revisar que tu solicitud siga esperando su Vo. Bo.</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Que Jesús dé su primer Vo. Bo. desde su computadora y vea la constancia con QR</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Reglas: llenar la pestaña "2. Preguntas"</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Datos: completar correo y jefe en la ficha de cada persona; altas y bajas en la pestaña "3. Personal"</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Arranque: quién anuncia, por qué medio, qué día, ¿todos o un área piloto?</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DESPUÉS</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Mandarle a Claude esta hoja llena para generar el SQL de altas</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>No hace falta enseñar todos los reportes. Lo importante hoy es que él lo use.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Alta,Corregir,Baja"</formula1>
+    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No,Pendiente"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -507,98 +669,855 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Pregunta</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Respuesta rápida</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Detalle / notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Vacaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>¿Las vacaciones vencen?</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Si vencen: ¿a los cuántos meses del aniversario? (la ley sugiere 6)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Si vencen: ¿desde qué fecha arranca la regla para lo ya acumulado?</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Flotantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>¿Cuántos días flotantes hay por año?</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>¿Los flotantes que no se usan se pierden en diciembre?</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Las 17 personas que no venían en el archivo de Sistemas: ¿son bajas?</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Fechas de ingreso de las 4 personas con correo que no están en la base</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Los 2 correos que dicen "ixtapluca": ¿cuál es el correcto?</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Vo. Bo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>¿Quién más de Gente y Cultura da Vo. Bo.? (para las solicitudes del propio Jesús)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Arranque</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>¿Quién anuncia el arranque?</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr"/>
+      <c r="D16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>¿Por qué medio?</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr"/>
+      <c r="D17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>¿Qué día arranca?</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>¿Todos o un área piloto primero?</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
+  <dataValidations count="13">
+    <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No,Lo confirma después"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"6 meses,12 meses,18 meses,Otro"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Hoy,1 de enero 2027,Otra fecha"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3,Otro"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Todas,Algunas,Ninguna"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Las da hoy,Las manda después"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Lo corrige hoy,Lo manda después"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Hay alguien,No hay nadie"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Jesús,Dirección,Uzziel"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Correo,WhatsApp,Junta,Varios"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Esta semana,Próxima semana,Otra fecha"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Todos,Área piloto"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Pregunta</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Respuesta</t>
+          <t>Una fila por persona. Alta = no está en la base · Corregir = está pero un dato está mal · Baja = ya no trabaja aquí.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>¿Cuántos días flotantes hay por año?</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr"/>
+          <t>Acción</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Nombre (APELLIDOS NOMBRES)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Fecha de ingreso</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Correo corporativo</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Puesto</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Área</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>No. de empleado</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Jefe directo</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>¿Los flotantes no usados se pierden en diciembre?</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr"/>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>PÉREZ LÓPEZ MARÍA</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>15/03/2022</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>maria.perez@financieracrediflexi.com</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Asesora de crédito</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Operaciones</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>1234</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>MONTELLANO JESÚS</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>EJEMPLO — borrar esta fila</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>¿Las vacaciones vencen? ¿A los cuántos meses del aniversario?</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr"/>
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="8" t="n"/>
+      <c r="C4" s="9" t="n"/>
+      <c r="D4" s="8" t="n"/>
+      <c r="E4" s="8" t="n"/>
+      <c r="F4" s="8" t="n"/>
+      <c r="G4" s="8" t="n"/>
+      <c r="H4" s="8" t="n"/>
+      <c r="I4" s="8" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Si vencen: ¿desde qué fecha arranca la regla para lo ya acumulado?</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr"/>
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Las 17 personas que no venían en el archivo de Sistemas: ¿son bajas?</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr"/>
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="9" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Fechas de ingreso de las 4 personas con correo que no están en la base</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr"/>
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Los dos correos que dicen "ixtapluca": ¿cuál es el correcto?</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr"/>
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>¿Quién anuncia el arranque, por qué medio y cuándo?</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr"/>
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="9" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>¿Quién más de Gente y Cultura da Vo. Bo.? (para las solicitudes del propio Jesús)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="I10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="9" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="9" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="n"/>
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="9" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
+      <c r="H18" s="8" t="n"/>
+      <c r="I18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+      <c r="H19" s="8" t="n"/>
+      <c r="I19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="8" t="n"/>
+      <c r="H21" s="8" t="n"/>
+      <c r="I21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="9" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="n"/>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="9" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="9" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="9" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="n"/>
+      <c r="H26" s="8" t="n"/>
+      <c r="I26" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="9" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
+      <c r="H27" s="8" t="n"/>
+      <c r="I27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="9" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
+      <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="8" t="n"/>
+      <c r="H29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="9" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
+      <c r="H30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="n"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="n"/>
+      <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="9" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="9" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="9" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="8" t="n"/>
+      <c r="H35" s="8" t="n"/>
+      <c r="I35" s="8" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
+      <c r="H36" s="8" t="n"/>
+      <c r="I36" s="8" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+      <c r="H37" s="8" t="n"/>
+      <c r="I37" s="8" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="9" t="n"/>
+      <c r="D38" s="8" t="n"/>
+      <c r="E38" s="8" t="n"/>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="8" t="n"/>
+      <c r="H38" s="8" t="n"/>
+      <c r="I38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="8" t="n"/>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="n"/>
+      <c r="H39" s="8" t="n"/>
+      <c r="I39" s="8" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="9" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="8" t="n"/>
+      <c r="H40" s="8" t="n"/>
+      <c r="I40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n"/>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="9" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="9" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="9" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+      <c r="H43" s="8" t="n"/>
+      <c r="I43" s="8" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="A3:A43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Alta,Corregir,Baja"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Fecha" error="Escribe la fecha como dd/mm/aaaa" type="date" operator="between">
+      <formula1>DATE(1980,1,1)</formula1>
+      <formula2>DATE(2030,12,31)</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(vacaciones): preguntas de la junta explícitas, con el porqué de cada una
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rsis6J1oMR6Czvco8XtVk
</commit_message>
<xml_diff>
--- a/docs/vacaciones/junta-montellano.xlsx
+++ b/docs/vacaciones/junta-montellano.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,6 +49,13 @@
     <font>
       <i val="1"/>
       <color rgb="00888888"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="00666666"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -105,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,6 +129,12 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -669,275 +682,575 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Preguntas para Jesús. Léelas tal cual (columna C). La columna D es solo para ti: por qué importa, por si te pregunta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Pregunta</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Respuesta rápida</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Detalle / notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Vacaciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="4" t="n">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Pregunta (dila tal cual)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Por qué la preguntamos (para ti)</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Notas / detalle</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Vencimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>¿Las vacaciones vencen?</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="4" t="n">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Vencimiento</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>¿Las vacaciones vencen si la persona no las toma?</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Hoy la base acumula los días sin límite: hay 450 días pendientes entre 45 personas y el Director General acumula 26. El sistema ya puede manejar vencimiento, pero solo él decide la regla.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Si vencen: ¿a los cuántos meses del aniversario? (la ley sugiere 6)</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Vencimiento</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Si vencen: ¿cuántos meses después del aniversario se pierden los días que no se tomaron?</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>La ley dice que las vacaciones deben darse dentro de los 6 meses siguientes al aniversario, pero cada empresa puede tener su política. Si dice "Otro", anota el número en Notas.</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="75" customHeight="1">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Si vencen: ¿desde qué fecha arranca la regla para lo ya acumulado?</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Vencimiento</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Si vencen: ¿a partir de qué fecha empezamos a aplicar la regla a los días que la gente ya tiene acumulados?</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Si la regla se aplica hacia atrás, mucha gente perdería días de golpe el mismo día que se active. Con una fecha de arranque, lo ya acumulado tiene el mismo plazo, contado desde esa fecha. Anota la fecha exacta en Notas.</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Flotantes</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="4" t="n">
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>¿Cuántos días flotantes hay por año?</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="4" t="n">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Flotantes</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>¿Cuántos días flotantes le corresponden a cada persona por año?</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Hoy el sistema cuenta los días flotantes pero no tiene tope: alguien podría pedir más de los que le tocan. Si dice "Otro", anota el número.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>¿Los flotantes que no se usan se pierden en diciembre?</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Personal</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Flotantes</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>¿Los días flotantes son los mismos para todos, o cambian según la antigüedad o el puesto?</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>El sistema maneja un solo número para todos. Si cambian según antigüedad o puesto, hay que ajustarlo: anota la regla exacta en Notas.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10" ht="48" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Las 17 personas que no venían en el archivo de Sistemas: ¿son bajas?</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11" ht="34" customHeight="1">
+          <t>Flotantes</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Si alguien no usa sus días flotantes en el año, ¿se pierden el 31 de diciembre o se pasan al año siguiente?</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>El sistema cuenta los flotantes por año calendario, de enero a diciembre. Si se pasan al siguiente año, hay que cambiarlo.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Fechas de ingreso de las 4 personas con correo que no están en la base</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="4" t="n">
+          <t>Flotantes</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>¿Una persona con menos de un año en la empresa puede usar días flotantes?</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Las vacaciones de ley empiezan al cumplir el primer año. Hoy el sistema deja pedir flotantes desde el primer día; si no debe ser así, hay que cambiarlo.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="75" customHeight="1">
+      <c r="A13" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Los 2 correos que dicen "ixtapluca": ¿cuál es el correcto?</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Vo. Bo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Hay 17 personas en tu base de vacaciones que no vienen en el archivo "Información para Sistemas". ¿Siguen trabajando aquí o ya son bajas?</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Si son bajas, se marcan como inactivas y dejan de contar. Si siguen, les falta correo y jefe para poder pedir vacaciones. Revisen la lista de nombres en la plataforma y anota las bajas en la pestaña 3.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>9</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>¿Quién más de Gente y Cultura da Vo. Bo.? (para las solicitudes del propio Jesús)</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Arranque</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Hay 4 personas que tienen correo de la empresa pero no aparecen en tu base de vacaciones. ¿Cuál es la fecha de ingreso de cada una?</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Sin fecha de ingreso el sistema no puede calcular sus días. Captúralas como "Alta" en la pestaña 3.</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Hay dos correos de asesoras de Ixtapaluca escritos sin la "a": asesor.ixtapluca1 (Viridiana Cabrera Flores) y asesor.ixtapluca3 (Ma. Inés Juárez Palma). Las demás de esa sucursal dicen "ixtapaluca". ¿Así se crearon esas cuentas en Google, o es un error al capturarlas en el archivo?</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Para entrar a pedir vacaciones, el correo en la base debe ser idéntico a su cuenta de Google. Si es error de captura, esas dos asesoras no podrán entrar hasta corregirlo. Si Jesús no sabe: preguntarle a quien administra las cuentas de Google, o a una de ellas con qué correo entra.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>¿Quién anuncia el arranque?</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17" ht="34" customHeight="1">
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Los correos de los asesores son por puesto (por ejemplo asesor.ixtapaluca1), no por persona. Cuando una asesora se va y entra otra al mismo puesto, ¿la nueva persona usa la misma cuenta de correo?</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Si se reutiliza la cuenta, en cada cambio hay que actualizar la base; si no, la persona nueva vería en "Mis vacaciones" los días de quien se fue.</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="48" customHeight="1">
       <c r="A17" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>¿Por qué medio?</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr"/>
-      <c r="D17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>¿Qué día arranca?</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19" ht="34" customHeight="1">
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Cuando alguien entra o sale de la empresa, ¿quién me avisa para darlo de alta o de baja en la plataforma?</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Hoy las altas se hacen por SQL (no hay pantalla). Hace falta saber quién avisa y por qué medio para que la base no se desactualice.</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Vo. Bo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>13</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>¿Todos o un área piloto primero?</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr"/>
-      <c r="D19" s="5" t="inlineStr"/>
+          <t>Vo. Bo.</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Cuando tú pidas vacaciones, el sistema no te deja aprobarte a ti mismo. ¿Quién más de Gente y Cultura puede dar el Vo. Bo. a tus solicitudes?</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Esa persona necesita cuenta y la bandera "Vacac." en el panel de administración. Anota su nombre en Notas.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Vo. Bo.</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>¿Quién es tu jefe directo, para que sea quien autorice tus vacaciones?</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Cada persona necesita su jefe directo en la base para que su solicitud llegue al jefe correcto. Anota el nombre en Notas.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Arranque</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Arranque</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>¿Quién manda el aviso de arranque al personal?</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Lo ideal es que salga de Gente y Cultura: es su proceso. Uzziel le pasa el texto redactado.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Arranque</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>¿Por qué medio avisamos al personal?</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Para preparar el texto en el formato correcto.</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Arranque</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>¿Qué día arrancamos?</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Anota la fecha exacta en Notas.</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Arranque</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>¿Arrancamos con todo el personal o primero con un área de prueba?</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Un área de prueba permite corregir detalles antes de abrirlo a todos. Si es área de prueba, anota cuál en Notas.</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Arranque</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Durante las primeras semanas, ¿sigues llevando tu Excel en paralelo o la plataforma lo reemplaza desde el primer día?</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Llevar los dos un tiempo da confianza, pero hay que acordar una fecha para dejar el Excel. Anota la fecha si la hay.</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A13:D13"/>
+  <mergeCells count="6">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
-  <dataValidations count="13">
-    <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No,Lo confirma después"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="19">
+    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí vencen,No vencen,Lo confirma después"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"6 meses,12 meses,18 meses,Otro"</formula1>
     </dataValidation>
-    <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Hoy,1 de enero 2027,Otra fecha"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Desde hoy,Desde el 1 de enero de 2027,Otra fecha"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,Otro"</formula1>
     </dataValidation>
-    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Todas,Algunas,Ninguna"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Iguales para todos,Según antigüedad,Según puesto"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Se pierden,Se pasan al siguiente año"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí puede,No puede"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Todas son bajas,Algunas son bajas,Todas siguen"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Las da hoy,Las manda después"</formula1>
     </dataValidation>
-    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Lo corrige hoy,Lo manda después"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Hay alguien,No hay nadie"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Así son las cuentas,Es error de captura,No sabe"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí, la misma cuenta,No, cuenta nueva,No sabe"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Jesús,Sistemas,Otra persona"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Hay alguien,No hay nadie más"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Lo dice hoy,Lo confirma después"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Jesús,Dirección,Uzziel"</formula1>
     </dataValidation>
-    <dataValidation sqref="C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Correo,WhatsApp,Junta,Varios"</formula1>
     </dataValidation>
-    <dataValidation sqref="C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Esta semana,Próxima semana,Otra fecha"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Todos,Área piloto"</formula1>
+    <dataValidation sqref="E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Esta semana,La próxima semana,Otra fecha"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Todo el personal,Área de prueba"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"En paralelo,Reemplaza desde el día uno"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>